<commit_message>
chore(students): add student 25 and update corrected emails in lists and sql scripts
</commit_message>
<xml_diff>
--- a/Alumnos_Diplomado_Septiembre_2026.xlsx
+++ b/Alumnos_Diplomado_Septiembre_2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Septiembre 2026" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,11 +397,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v xml:space="preserve">﻿No</v>
+        <v>No</v>
       </c>
       <c r="B1" t="str">
         <v>Nombre Completo</v>
@@ -442,7 +442,7 @@
         <v>Jeniffer Vanesa Salguero García</v>
       </c>
       <c r="C2" t="str">
-        <v>jeniffersalgueroz21@gmail.com</v>
+        <v>jeniffersalguero21@gmail.com</v>
       </c>
       <c r="D2" t="str">
         <v>IAV2026*6948</v>
@@ -1107,7 +1107,7 @@
         <v>Beatriz Elena Ibarra Aguirre</v>
       </c>
       <c r="C21" t="str">
-        <v>elenaibarra1545@gmail.com</v>
+        <v>elena.ibarra1595@gmail.com</v>
       </c>
       <c r="D21" t="str">
         <v>IAV2026*4097</v>
@@ -1274,9 +1274,44 @@
         <v>https://iavolution.academy</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Diana Stephanie Sandoval Aguilar</v>
+      </c>
+      <c r="C26" t="str">
+        <v>iam.dianasandoval@gmail.com</v>
+      </c>
+      <c r="D26" t="str">
+        <v>IAV2026*1598</v>
+      </c>
+      <c r="E26" t="str">
+        <v>7015-1598</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Tecnico en Marketing</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Cancio Asosiados</v>
+      </c>
+      <c r="H26" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Diplomado en Automatización de Procesos con IA</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Septiembre 2026</v>
+      </c>
+      <c r="K26" t="str">
+        <v>https://iavolution.academy</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>